<commit_message>
BGS98-5: questions on BGS98 harmonisation in the analyst files
</commit_message>
<xml_diff>
--- a/analyst/Ines/rmonize/data_dictionary/DD_BGS98_INES.xlsx
+++ b/analyst/Ines/rmonize/data_dictionary/DD_BGS98_INES.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\use-cases-harmonisation\analyst\Ines\rmonize\data_dictionary\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\analyst\Ines\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4ED2C2A-1CEF-4407-BC88-B65D6428E57A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42047779-2718-4415-962F-738BB4E7A477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -164,7 +164,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -193,6 +193,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -214,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -227,9 +235,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -532,13 +544,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="49.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="49.7109375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -552,7 +564,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>12</v>
       </c>
@@ -563,7 +575,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
         <v>13</v>
       </c>
@@ -574,7 +586,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>6</v>
       </c>
@@ -585,8 +597,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B5" s="5" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="3" t="s">
@@ -596,7 +608,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>17</v>
       </c>
@@ -607,7 +619,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>20</v>
       </c>
@@ -618,7 +630,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>19</v>
       </c>
@@ -629,7 +641,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>7</v>
       </c>
@@ -640,7 +652,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>21</v>
       </c>
@@ -651,7 +663,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>24</v>
       </c>
@@ -662,7 +674,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>26</v>
       </c>
@@ -673,7 +685,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>27</v>
       </c>
@@ -684,7 +696,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>28</v>
       </c>
@@ -695,7 +707,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>29</v>
       </c>
@@ -706,7 +718,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>32</v>
       </c>
@@ -717,18 +729,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" t="s">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B17" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D17" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>38</v>
       </c>
@@ -739,18 +751,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19" t="s">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B19" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="7" t="s">
         <v>41</v>
       </c>
       <c r="D19" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>42</v>
       </c>
@@ -769,9 +781,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
BGS98-INES DPEs and DD.
</commit_message>
<xml_diff>
--- a/analyst/Ines/rmonize/data_dictionary/DD_BGS98_INES.xlsx
+++ b/analyst/Ines/rmonize/data_dictionary/DD_BGS98_INES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\use-cases-harmonisation\analyst\Ines\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC2A89D3-7467-4BCC-A57D-BB66AF7970FB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4894285A-DA3B-4D3F-9F0A-5BD2E020E8F3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="52">
   <si>
     <t>index</t>
   </si>
@@ -152,6 +152,36 @@
   </si>
   <si>
     <t>UShuef_FUP</t>
+  </si>
+  <si>
+    <t>GFS</t>
+  </si>
+  <si>
+    <t>ges.FS (g/d)</t>
+  </si>
+  <si>
+    <t>GFU</t>
+  </si>
+  <si>
+    <t>unges.FS (g/d)</t>
+  </si>
+  <si>
+    <t>GKD</t>
+  </si>
+  <si>
+    <t>Disacch (g/d)</t>
+  </si>
+  <si>
+    <t>GKM</t>
+  </si>
+  <si>
+    <t>Monosacch (g/d)</t>
+  </si>
+  <si>
+    <t>AGE_ANTH_FUP</t>
+  </si>
+  <si>
+    <t>Age at anthropometric measurement at follow-up [years]</t>
   </si>
 </sst>
 </file>
@@ -562,10 +592,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="49.7109375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
@@ -778,6 +808,61 @@
         <v>36</v>
       </c>
       <c r="D19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>46</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D23" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>